<commit_message>
Adiciona cabeçalho de identificação (logo + dados) na tela de Proposta
PropostaSimulacaoPanel.tsx ganha um cabeçalho sempre visível (na simulação
e depois de confirmada) com a logo da Navegantes e os dados de
identificação no mesmo layout da aba "Requerimento 2026" do Excel de
referência: nome do aluno, série, sexo, data de nascimento e nome do
Responsável Financeiro (prioriza o vínculo TIPO "Financeiro", depois
"Legal e Financeiro", quando o aluno tem mais de um responsável vinculado).
Vale nos dois fluxos que reaproveitam o painel (Fazer Proposta e Gerador
de Proposta). Puramente visual -- nenhuma lógica de cálculo, endpoint ou
regra de desconto foi alterada.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/01_CADASTROS.xlsx
+++ b/backend/data/01_CADASTROS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="246">
   <si>
     <t>ID_ALUNO</t>
   </si>
@@ -107,10 +107,31 @@
     <t>TELEFONE</t>
   </si>
   <si>
+    <t>RES_000001</t>
+  </si>
+  <si>
+    <t>Responsável Financeiro Acentuação Ção</t>
+  </si>
+  <si>
+    <t>000.000.000-00</t>
+  </si>
+  <si>
+    <t>teste@teste.com</t>
+  </si>
+  <si>
+    <t>11999999999</t>
+  </si>
+  <si>
     <t>ID_ALUNO_RESPONSAVEL</t>
   </si>
   <si>
     <t>TIPO</t>
+  </si>
+  <si>
+    <t>AR_000001</t>
+  </si>
+  <si>
+    <t>Financeiro</t>
   </si>
   <si>
     <t>ID_ANO_LETIVO</t>
@@ -1246,7 +1267,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1268,19 +1289,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
@@ -1299,7 +1320,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1310,10 +1331,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1321,10 +1342,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="B3" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1332,10 +1353,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="B4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1343,10 +1364,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B5" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1354,10 +1375,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="B6" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1365,10 +1386,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="B7" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1376,10 +1397,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B8" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -1387,10 +1408,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="B9" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1398,10 +1419,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B10" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -1409,10 +1430,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="B11" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -1420,10 +1441,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="B12" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="C12" t="b">
         <v>1</v>
@@ -1431,10 +1452,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B13" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
@@ -1442,10 +1463,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B14" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C14" t="b">
         <v>1</v>
@@ -1453,10 +1474,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B15" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C15" t="b">
         <v>1</v>
@@ -1464,10 +1485,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B16" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
@@ -1475,10 +1496,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B17" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1486,10 +1507,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="B18" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C18" t="b">
         <v>1</v>
@@ -1497,10 +1518,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B19" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C19" t="b">
         <v>1</v>
@@ -1508,10 +1529,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B20" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C20" t="b">
         <v>1</v>
@@ -1519,10 +1540,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="B21" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
       <c r="C21" t="b">
         <v>1</v>
@@ -1530,10 +1551,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B22" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C22" t="b">
         <v>1</v>
@@ -1541,10 +1562,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="B23" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
@@ -1552,10 +1573,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="B24" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="C24" t="b">
         <v>1</v>
@@ -1563,10 +1584,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B25" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
@@ -1574,10 +1595,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="B26" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="C26" t="b">
         <v>1</v>
@@ -1585,10 +1606,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="B27" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="C27" t="b">
         <v>1</v>
@@ -1596,10 +1617,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B28" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C28" t="b">
         <v>1</v>
@@ -1607,10 +1628,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="B29" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="C29" t="b">
         <v>1</v>
@@ -1618,10 +1639,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="B30" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C30" t="b">
         <v>1</v>
@@ -1629,10 +1650,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B31" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="C31" t="b">
         <v>0</v>
@@ -1640,10 +1661,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="B32" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="C32" t="b">
         <v>1</v>
@@ -1651,10 +1672,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B33" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1662,10 +1683,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B34" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="C34" t="b">
         <v>1</v>
@@ -1673,10 +1694,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="B35" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="C35" t="b">
         <v>1</v>
@@ -1684,10 +1705,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B36" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C36" t="b">
         <v>1</v>
@@ -1695,10 +1716,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="C37" t="b">
         <v>1</v>
@@ -1706,10 +1727,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="C38" t="b">
         <v>1</v>
@@ -1717,10 +1738,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B39" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C39" t="b">
         <v>1</v>
@@ -1728,10 +1749,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B40" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="C40" t="b">
         <v>1</v>
@@ -1739,10 +1760,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C41" t="b">
         <v>1</v>
@@ -1750,10 +1771,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="B42" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="C42" t="b">
         <v>1</v>
@@ -1761,10 +1782,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B43" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="C43" t="b">
         <v>1</v>
@@ -1783,7 +1804,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1794,10 +1815,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1805,10 +1826,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B3" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1816,10 +1837,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="B4" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1827,10 +1848,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="B5" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1838,10 +1859,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
       <c r="B6" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1849,10 +1870,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="B7" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1871,7 +1892,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1888,7 +1909,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1909,6 +1930,26 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1919,12 +1960,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -1933,10 +1974,27 @@
         <v>23</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E2" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1974,10 +2032,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>10</v>
@@ -1985,7 +2043,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <v>2026</v>
@@ -2013,10 +2071,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
@@ -2024,13 +2082,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -2038,13 +2096,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D3" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -2052,13 +2110,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -2066,13 +2124,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -2080,13 +2138,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -2094,13 +2152,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -2108,13 +2166,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -2122,13 +2180,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -2136,13 +2194,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -2150,13 +2208,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B11" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -2164,13 +2222,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -2178,13 +2236,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -2192,13 +2250,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B14" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -2206,13 +2264,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B15" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
@@ -2220,13 +2278,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -2234,13 +2292,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="D17" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -2248,13 +2306,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -2262,13 +2320,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -2276,13 +2334,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -2290,13 +2348,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -2304,13 +2362,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D22" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -2318,13 +2376,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B23" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
@@ -2332,13 +2390,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
@@ -2346,13 +2404,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
@@ -2363,10 +2421,10 @@
         <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D26" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
@@ -2374,13 +2432,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -2388,13 +2446,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="D28" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -2402,13 +2460,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B29" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -2419,10 +2477,10 @@
         <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D30" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -2430,13 +2488,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B31" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D31" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -2444,13 +2502,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B32" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D32" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -2458,13 +2516,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E33" t="b">
         <v>1</v>
@@ -2472,13 +2530,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D34" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
@@ -2486,13 +2544,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B35" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D35" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -2500,13 +2558,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B36" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D36" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -2514,13 +2572,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B37" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D37" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
@@ -2528,13 +2586,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B38" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="D38" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
@@ -2542,13 +2600,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B39" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
@@ -2556,13 +2614,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B40" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="D40" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
@@ -2570,13 +2628,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B41" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D41" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
@@ -2584,13 +2642,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D42" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
@@ -2598,13 +2656,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B43" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="D43" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -2612,13 +2670,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B44" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="D44" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
@@ -2626,13 +2684,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B45" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
@@ -2640,13 +2698,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B46" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="D46" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
@@ -2654,13 +2712,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B47" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D47" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
@@ -2668,13 +2726,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B48" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="D48" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E48" t="b">
         <v>1</v>
@@ -2682,13 +2740,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B49" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="D49" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E49" t="b">
         <v>1</v>
@@ -2696,13 +2754,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B50" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D50" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E50" t="b">
         <v>1</v>
@@ -2710,13 +2768,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B51" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="D51" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -2724,13 +2782,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B52" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="D52" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="E52" t="b">
         <v>1</v>
@@ -2761,10 +2819,10 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
@@ -2783,7 +2841,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2792,7 +2850,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
@@ -2825,7 +2883,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -2836,7 +2894,7 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualiza snapshot de dados reais (interações/testes desde o último commit)
Sem mudança de código -- só o estado atual de backend/data/ depois de
verificações manuais na tela de Proposta (responsável de teste criado e
já excluído logicamente, propostas de teste criadas ao validar o wizard).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/01_CADASTROS.xlsx
+++ b/backend/data/01_CADASTROS.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="248">
   <si>
     <t>ID_ALUNO</t>
   </si>
@@ -95,6 +95,15 @@
     <t>TUN_000002</t>
   </si>
   <si>
+    <t>ALU_000003</t>
+  </si>
+  <si>
+    <t>Joaquim</t>
+  </si>
+  <si>
+    <t>SER_000013</t>
+  </si>
+  <si>
     <t>ID_RESPONSAVEL</t>
   </si>
   <si>
@@ -216,9 +225,6 @@
   </si>
   <si>
     <t>1º Período C</t>
-  </si>
-  <si>
-    <t>SER_000013</t>
   </si>
   <si>
     <t>2º Período A</t>
@@ -1143,7 +1149,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1252,6 +1258,41 @@
       </c>
       <c r="K3" t="b">
         <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2">
+        <v>44209</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="2">
+        <v>46278</v>
+      </c>
+      <c r="K4" t="b">
+        <v>1</v>
+      </c>
+      <c r="L4" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -1267,7 +1308,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1289,19 +1330,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
@@ -1320,7 +1361,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1331,10 +1372,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B2" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1342,10 +1383,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1353,10 +1394,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1364,10 +1405,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1375,10 +1416,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1386,10 +1427,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B7" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1397,10 +1438,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B8" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -1408,10 +1449,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1419,10 +1460,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B10" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -1430,10 +1471,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -1441,10 +1482,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B12" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C12" t="b">
         <v>1</v>
@@ -1452,10 +1493,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B13" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
@@ -1463,10 +1504,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B14" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C14" t="b">
         <v>1</v>
@@ -1474,10 +1515,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B15" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C15" t="b">
         <v>1</v>
@@ -1485,10 +1526,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B16" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C16" t="b">
         <v>1</v>
@@ -1496,10 +1537,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B17" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
@@ -1507,10 +1548,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B18" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C18" t="b">
         <v>1</v>
@@ -1518,10 +1559,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B19" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C19" t="b">
         <v>1</v>
@@ -1529,10 +1570,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C20" t="b">
         <v>1</v>
@@ -1540,10 +1581,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B21" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C21" t="b">
         <v>1</v>
@@ -1551,10 +1592,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B22" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C22" t="b">
         <v>1</v>
@@ -1562,10 +1603,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B23" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
@@ -1573,10 +1614,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B24" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C24" t="b">
         <v>1</v>
@@ -1584,10 +1625,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B25" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
@@ -1595,10 +1636,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B26" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C26" t="b">
         <v>1</v>
@@ -1606,10 +1647,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B27" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C27" t="b">
         <v>1</v>
@@ -1617,10 +1658,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B28" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C28" t="b">
         <v>1</v>
@@ -1628,10 +1669,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B29" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C29" t="b">
         <v>1</v>
@@ -1639,10 +1680,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B30" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C30" t="b">
         <v>1</v>
@@ -1650,10 +1691,10 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B31" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C31" t="b">
         <v>0</v>
@@ -1661,10 +1702,10 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B32" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C32" t="b">
         <v>1</v>
@@ -1672,10 +1713,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B33" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C33" t="b">
         <v>1</v>
@@ -1683,10 +1724,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B34" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C34" t="b">
         <v>1</v>
@@ -1694,10 +1735,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B35" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C35" t="b">
         <v>1</v>
@@ -1705,10 +1746,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B36" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C36" t="b">
         <v>1</v>
@@ -1716,10 +1757,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B37" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C37" t="b">
         <v>1</v>
@@ -1727,10 +1768,10 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B38" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C38" t="b">
         <v>1</v>
@@ -1738,10 +1779,10 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B39" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C39" t="b">
         <v>1</v>
@@ -1749,10 +1790,10 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B40" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C40" t="b">
         <v>1</v>
@@ -1760,10 +1801,10 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B41" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C41" t="b">
         <v>1</v>
@@ -1771,10 +1812,10 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B42" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="C42" t="b">
         <v>1</v>
@@ -1782,10 +1823,10 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B43" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C43" t="b">
         <v>1</v>
@@ -1804,7 +1845,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1815,10 +1856,10 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -1826,10 +1867,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>
@@ -1837,10 +1878,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C4" t="b">
         <v>1</v>
@@ -1848,10 +1889,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B5" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -1859,10 +1900,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B6" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -1870,10 +1911,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B7" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -1892,7 +1933,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -1914,19 +1955,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>10</v>
@@ -1934,19 +1975,19 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -1965,16 +2006,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
@@ -1982,16 +2023,16 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
         <v>18</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="D2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -2032,10 +2073,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>10</v>
@@ -2043,7 +2084,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <v>2026</v>
@@ -2071,10 +2112,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>39</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>36</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
@@ -2082,13 +2123,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E2" t="b">
         <v>1</v>
@@ -2096,13 +2137,13 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D3" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E3" t="b">
         <v>1</v>
@@ -2110,13 +2151,13 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E4" t="b">
         <v>1</v>
@@ -2124,13 +2165,13 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -2138,13 +2179,13 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E6" t="b">
         <v>1</v>
@@ -2152,13 +2193,13 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -2166,13 +2207,13 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -2180,13 +2221,13 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -2194,13 +2235,13 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -2208,13 +2249,13 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="D11" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -2222,13 +2263,13 @@
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -2236,13 +2277,13 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -2250,13 +2291,13 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
       <c r="B14" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D14" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -2264,13 +2305,13 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
@@ -2278,13 +2319,13 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D16" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -2292,13 +2333,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D17" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -2306,13 +2347,13 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D18" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -2320,13 +2361,13 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D19" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E19" t="b">
         <v>1</v>
@@ -2334,13 +2375,13 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B20" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D20" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E20" t="b">
         <v>1</v>
@@ -2348,13 +2389,13 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B21" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E21" t="b">
         <v>1</v>
@@ -2362,13 +2403,13 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B22" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D22" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E22" t="b">
         <v>1</v>
@@ -2376,13 +2417,13 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B23" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E23" t="b">
         <v>1</v>
@@ -2390,13 +2431,13 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D24" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E24" t="b">
         <v>1</v>
@@ -2404,13 +2445,13 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D25" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
@@ -2421,10 +2462,10 @@
         <v>15</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D26" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E26" t="b">
         <v>1</v>
@@ -2432,13 +2473,13 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B27" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D27" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E27" t="b">
         <v>1</v>
@@ -2446,13 +2487,13 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B28" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D28" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E28" t="b">
         <v>1</v>
@@ -2460,13 +2501,13 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B29" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D29" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E29" t="b">
         <v>1</v>
@@ -2477,10 +2518,10 @@
         <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D30" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E30" t="b">
         <v>1</v>
@@ -2488,13 +2529,13 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B31" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D31" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E31" t="b">
         <v>1</v>
@@ -2502,13 +2543,13 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B32" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="D32" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -2516,13 +2557,13 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D33" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E33" t="b">
         <v>1</v>
@@ -2530,13 +2571,13 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D34" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E34" t="b">
         <v>1</v>
@@ -2544,13 +2585,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D35" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E35" t="b">
         <v>1</v>
@@ -2558,13 +2599,13 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B36" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D36" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E36" t="b">
         <v>1</v>
@@ -2572,13 +2613,13 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B37" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D37" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E37" t="b">
         <v>1</v>
@@ -2586,13 +2627,13 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B38" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D38" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E38" t="b">
         <v>1</v>
@@ -2600,13 +2641,13 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B39" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D39" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
@@ -2614,13 +2655,13 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B40" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D40" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
@@ -2628,13 +2669,13 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B41" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D41" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
@@ -2642,13 +2683,13 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B42" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="D42" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
@@ -2656,13 +2697,13 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B43" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D43" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -2670,13 +2711,13 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B44" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D44" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
@@ -2684,13 +2725,13 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B45" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D45" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
@@ -2698,13 +2739,13 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B46" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="D46" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
@@ -2712,13 +2753,13 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B47" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D47" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
@@ -2726,13 +2767,13 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B48" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D48" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E48" t="b">
         <v>1</v>
@@ -2740,13 +2781,13 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B49" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D49" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E49" t="b">
         <v>1</v>
@@ -2754,13 +2795,13 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B50" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D50" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E50" t="b">
         <v>1</v>
@@ -2768,13 +2809,13 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B51" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D51" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -2782,13 +2823,13 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B52" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D52" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="E52" t="b">
         <v>1</v>
@@ -2819,10 +2860,10 @@
         <v>6</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>10</v>
@@ -2841,7 +2882,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -2850,7 +2891,7 @@
         <v>4</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>10</v>
@@ -2883,7 +2924,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C2" t="b">
         <v>1</v>
@@ -2894,7 +2935,7 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C3" t="b">
         <v>1</v>

</xml_diff>